<commit_message>
Refactored Stage 2 with Wards'clustering plus MRT. Added HZD in stage 1.
</commit_message>
<xml_diff>
--- a/results/02_taxa_assemblage/MRT_Method/cluster_classifier/tables/mrt_confusion_matrix.xlsx
+++ b/results/02_taxa_assemblage/MRT_Method/cluster_classifier/tables/mrt_confusion_matrix.xlsx
@@ -425,65 +425,105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ward_Cluster</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="n">
-        <v>3</v>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>% Correct</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cluster C1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Cluster C2</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Cluster C3</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>1</v>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Cluster C1</t>
+        </is>
       </c>
       <c r="B2" t="n">
+        <v>57</v>
+      </c>
+      <c r="C2" t="n">
         <v>12</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>5</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>2</v>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Cluster C2</t>
+        </is>
       </c>
       <c r="B3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C3" t="n">
         <v>0</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>14</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>3</v>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Cluster C3</t>
+        </is>
       </c>
       <c r="B4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" t="n">
         <v>2</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>7</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D5" t="n">
+        <v>26</v>
+      </c>
+      <c r="E5" t="n">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>